<commit_message>
Update docs and examples for source_ref expressions, row_filter, date_format
Docs:
- AGENTS.md: added expected row counts for examples 16 (4) and 17 (18)
- CONFIG_AUTHORING_GUIDE.md: expanded source_ref section with const:/fn:/expr: formats, operator tables, NULL handling, examples; added row_filter and date_format to sheet_config/column_config tables
- CONFIG_RULES.md: added row_filter to sheet_config table, expanded source_ref description with all four formats, added date_format to column_config table
</commit_message>
<xml_diff>
--- a/examples/01_simple/sales_config.xlsx
+++ b/examples/01_simple/sales_config.xlsx
@@ -4,7 +4,7 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="target_config" sheetId="1" state="visible" r:id="rId1"/>
@@ -78,9 +78,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -333,6 +335,23 @@
 Example: food_delivery</t>
       </text>
     </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t xml:space="preserve">where (optional)
+Row filter — only load rows that match this condition. Rows that don't match are silently skipped.
+Syntax: {COL_LETTER} operator value
+  Operators: =, !=, &gt;, &lt;, &gt;=, &lt;=, contains, not_contains, is_empty, is_not_empty
+  Combine with AND / OR
+Examples:
+  {D} &gt; 0                    (only rows where column D &gt; 0)
+  {A} != ""                  (skip empty rows in column A)
+  {B} = "Active"             (only Active rows)
+  {D} &gt; 0 AND {E} != "NA"   (two conditions)
+  {A} is_not_empty           (skip blank rows)
+Allowed: {COL} op value [AND/OR ...]; blank = load all rows
+Example: </t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -355,10 +374,30 @@
     <comment ref="B1" authorId="0" shapeId="0">
       <text>
         <t>source_ref (required)
-Which Excel column letter to read FROM the source file. The parser reads by column position, NOT by header text.
-Example: if 'Order ID' is in column A → 'col:A'. If 'Amount' is in column D → 'col:D'. Wide sheets: column 30 = 'col:AD'.
-IMPORTANT: if the supplier inserts a new column, every letter after it shifts. Re-check all source_ref values when that happens.
-Allowed: col:&lt;letter&gt; (e.g. col:A, col:B, col:AM). No row numbers, no ranges
+Where to get the value for this column. Four formats:
+1. Column reference: 'col:&lt;letter&gt;' — reads from the source file by position, NOT by header text. Example: col:A, col:D, col:AM.
+2. Constant value: 'const:&lt;value&gt;' — fills every row with a fixed value. Example: const:adarsh, const:100.
+3. Computed value: 'fn:&lt;name&gt;' — fills every row with a value computed at load time. Available functions:
+  fn:now       — current timestamp (timestamp, text)
+  fn:today     — current date (date, text)
+  fn:uuid      — random UUID per row (text)
+  fn:file_name — source file name (text)
+  fn:sequence  — counter 1,2,3... per table (integer, numeric, text)
+4. Expression: 'expr:&lt;expression&gt;' — computes a value from other columns, constants, functions and literals. Use {X} to reference Excel column X.
+  Operators: + - * / (numeric), &amp; (string concatenation)
+  Grouping: parentheses ( ) to override precedence
+  Unary minus: -{A} to negate a value
+  NULL handling: arithmetic with NULL -&gt; NULL (like SQL)
+  Examples:
+    expr:{D} + {E}             (sum two columns)
+    expr:({A} + {B}) * {C}     (grouped arithmetic)
+    expr:-{D}                  (negate a value)
+    expr:{A} &amp; " - " &amp; {C}    (concatenate with separator)
+    expr:{D} * 0.18            (calculate 18% tax)
+All results are cast to the column's data_type. 'script' and
+'null_default' apply after the expression result is cast.
+IMPORTANT: if the supplier inserts a new column, every letter after it shifts. Re-check all col: and expr: source_ref values when that happens.
+Allowed: col:&lt;letter&gt;, const:&lt;value&gt;, fn:&lt;name&gt;, or expr:&lt;expression&gt;
 Example: col:A</t>
       </text>
     </comment>
@@ -740,23 +779,23 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" style="3" min="1" max="1"/>
+    <col width="22" customWidth="1" style="3" min="2" max="2"/>
+    <col width="90" customWidth="1" style="3" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -856,70 +895,76 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="4"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="8"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" style="3" min="1" max="4"/>
+    <col width="14" customWidth="1" style="3" min="2" max="2"/>
+    <col width="14" customWidth="1" style="3" min="3" max="3"/>
+    <col width="14" customWidth="1" style="3" min="4" max="4"/>
+    <col width="18" customWidth="1" style="3" min="5" max="5"/>
+    <col width="16" customWidth="1" style="3" min="6" max="6"/>
+    <col width="14" customWidth="1" style="3" min="7" max="8"/>
+    <col width="14" customWidth="1" style="3" min="8" max="8"/>
+    <col width="15" customWidth="1" style="3" min="9" max="9"/>
+    <col width="14" customWidth="1" style="3" min="10" max="10"/>
+    <col width="14" customWidth="1" style="3" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>table_name</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>sheet_name</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>layout</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>header_row</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>data_start_row</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>data_end_row</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>domain</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>where</t>
         </is>
       </c>
     </row>
@@ -963,6 +1008,11 @@
       <c r="J2" t="inlineStr">
         <is>
           <t>sales</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>{D} &gt; 1000</t>
         </is>
       </c>
     </row>
@@ -983,84 +1033,83 @@
   <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="2"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="8"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" style="3" min="1" max="2"/>
+    <col width="14" customWidth="1" style="3" min="2" max="2"/>
+    <col width="17" customWidth="1" style="3" min="3" max="3"/>
+    <col width="15" customWidth="1" style="3" min="4" max="4"/>
+    <col width="14" customWidth="1" style="3" min="5" max="7"/>
+    <col width="14" customWidth="1" style="3" min="6" max="6"/>
+    <col width="14" customWidth="1" style="3" min="7" max="7"/>
+    <col width="16" customWidth="1" style="3" min="8" max="8"/>
+    <col width="14" customWidth="1" style="3" min="9" max="9"/>
+    <col width="16" customWidth="1" style="3" min="10" max="10"/>
+    <col width="15" customWidth="1" style="3" min="11" max="11"/>
+    <col width="14" customWidth="1" style="3" min="12" max="14"/>
+    <col width="14" customWidth="1" style="3" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>table_name</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>source_ref</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>source_header</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>column_name</t>
         </is>
       </c>
-      <c r="E1" s="5" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>nullable</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>is_key</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>column_order</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>references</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>null_default</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="L1" s="5" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>script</t>
         </is>
@@ -1261,6 +1310,7 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="15" customHeight="1" s="3"/>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1278,59 +1328,59 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" style="3" min="1" max="1"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
+    <col width="58" customWidth="1" style="3" min="3" max="3"/>
+    <col width="58" customWidth="1" style="3" min="4" max="4"/>
+    <col width="30" customWidth="1" style="3" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>target_config - where the rows are pushed</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>header / setting</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>what it means</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>allowed values</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>example</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>target</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Which database to push into.
   'sqlite'  → a local file (good for testing and small datasets)
@@ -1338,127 +1388,127 @@
 Example: use 'sqlite' while developing, then switch to 'postgres' for production.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>sqlite | postgres (default sqlite)</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>postgres</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>database</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>SQLite: the file path (e.g. 'loaded.db' creates a file in the working directory).
 PostgreSQL: the database NAME (e.g. 'excel_parser').
 Leave blank to take it from the command line (--database) or the PGDATABASE environment variable.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>any path for sqlite; a plain name for postgres</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>excel_parser</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>db_schema</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>PostgreSQL schema to load into. Created automatically if it does not exist.
 Example: 'staging' puts all tables under the 'staging' schema. Blank = the 'public' schema. Ignored by SQLite (no schemas).</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>plain name; blank = public. Ignored by SQLite</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>staging</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>table_prefix</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>A prefix added to every table name.
 Example: if table_prefix='stg_' and table_name='orders', the physical table is 'stg_orders'. Useful for separating staging from production tables in the same schema.
 Blank = no prefix (default).</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>plain name fragment; blank = no prefix</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>(blank)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>id_type</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>How primary keys and file_id are generated.
   'integer' → auto-incrementing numbers (1, 2, 3...) — simpler, default.
   'uuid'    → random UUIDs per row — use when merging data from multiple sources where integer IDs would collide.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>integer | uuid (default integer)</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
@@ -1475,118 +1525,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" style="3" min="1" max="1"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
+    <col width="58" customWidth="1" style="3" min="3" max="3"/>
+    <col width="58" customWidth="1" style="3" min="4" max="4"/>
+    <col width="30" customWidth="1" style="3" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>sheet_config - one row per block to read</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>header / setting</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>what it means</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>allowed values</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>example</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>table_name</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>The database table name for this block. The physical table becomes &lt;table_prefix&gt;&lt;table_name&gt;.
 Example: if your source has an 'Orders' tab, you might name it 'orders'. Two blocks on the same sheet need different names — e.g. 'card_payments' and 'cash_payments' for two sections on a 'Payments' tab.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>lowercase letters, digits, underscore; unique in the workbook; max 63 chars</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>orders</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>sheet_name</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>The exact tab name in the SOURCE workbook. Must match character for character — copy-paste it from the tab to avoid typos.
 Example: if the tab is called 'Order Level', type exactly 'Order Level'. Excel truncates long tab names (e.g. 'Growth Investments and Other De'), so copy the truncated name.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>exact tab name from the source file</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Order Level</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>layout</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Describes the shape of the data block:
   'table' = a header row (e.g. row 1) followed by data rows below it.
@@ -1594,208 +1644,245 @@
 Example: a list of orders with columns Date, Customer, Amount → 'table'. A summary block with 'Total Orders: 42' on one row → 'key_value'.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>table | key_value</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>table</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>header_row</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>The row number that contains column headers (e.g. 'Date', 'Customer', 'Amount'). Not read as data — only recorded in the audit log.
 Example: if row 1 has headers and data starts at row 2, set header_row=1. Leave blank for key_value layout.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>whole number, 1-based as shown in Excel; blank for key_value</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>data_start_row</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>The FIRST row of actual data (not the header, not a title row). Look at the row numbers in Excel.
 Example: if row 1 is headers and data starts at row 2, set data_start_row=2. If there is a title on rows 1–3, headers on row 4, and data from row 5, set data_start_row=5.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>whole number, must be below the header/title row</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>data_end_row</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>The LAST row of data. Set this when there are totals, notes, or another data block below.
 Example: data in rows 2–50, then a 'Grand Total' on row 51 → set data_end_row=50. If another block starts at row 55, fence this one off at row 50.
 Leave blank to read to the last non-empty row in the sheet.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>whole number &gt;= data_start_row; blank = read to the last used row</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>(blank)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>row_filter</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Skip rows that don't match this condition.
+Use col:LETTER to reference a cell (same as source_ref), then an operator and a value.
+Operators:
+  =  !=  &gt;  &lt;  &gt;=  &lt;=        compare text or numbers
+  contains  not_contains     text search inside the cell
+  is_empty  is_not_empty     check for blank cells (no value needed)
+Examples:
+  col:A is_not_empty              skip blank rows
+  col:D &gt; 0                       only positive amounts
+  col:B = "Delivered"             only delivered orders
+  col:C != "Cancelled"            exclude cancelled
+  col:E contains "swiggy"         cell contains the word
+  col:D &gt; 100 AND col:F != "NA"   combine two conditions
+  col:A = "Active" OR col:A = "Pending"   either status
+Leave blank to load all rows (default).</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>col:LETTER op value [AND/OR ...]; blank = all rows</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Y = this block is processed (table created, data loaded).
 N = completely skipped — use this to park a block you do not want right now without deleting the row.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Y | N</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>A human-readable description of what this table contains. Written as a COMMENT ON TABLE in PostgreSQL so BI tools and AI agents can discover meaning.
 Example: 'Order-level payout details from the Swiggy annexure'</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>any text</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Order-level payout details from the delivery platform</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>A business category tag. Prepended to the table comment as [domain].
 Example: 'finance', 'orders', 'inventory', 'hr'</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>any text</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>food_delivery</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Free text for your own use. Copied into the generated SQL as a comment.</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>any text</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>invoice lines, one row per invoice</t>
         </is>
@@ -1812,176 +1899,196 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="58" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" style="3" min="1" max="1"/>
+    <col width="10" customWidth="1" style="3" min="2" max="2"/>
+    <col width="58" customWidth="1" style="3" min="3" max="3"/>
+    <col width="58" customWidth="1" style="3" min="4" max="4"/>
+    <col width="30" customWidth="1" style="3" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>column_config - one row per database column</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>header / setting</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>required</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>what it means</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
         <is>
           <t>allowed values</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>example</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>table_name</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Which block (from sheet_config) this column belongs to.
 Example: if you defined a block called 'orders' in sheet_config, every column row for that block has table_name='orders'.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>must match a table_name on sheet_config</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>orders</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>source_ref</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Which Excel column letter to read FROM the source file. The parser reads by column position, NOT by header text.
-Example: if 'Order ID' is in column A → 'col:A'. If 'Amount' is in column D → 'col:D'. Wide sheets: column 30 = 'col:AD'.
-IMPORTANT: if the supplier inserts a new column, every letter after it shifts. Re-check all source_ref values when that happens.</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>col:&lt;letter&gt; (e.g. col:A, col:B, col:AM). No row numbers, no ranges</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Where to get the value for this column. Four formats:
+1. Column reference: 'col:&lt;letter&gt;' — reads from the source file by position, NOT by header text. Example: col:A, col:D, col:AM.
+2. Constant value: 'const:&lt;value&gt;' — fills every row with a fixed value. Example: const:adarsh, const:100.
+3. Computed value: 'fn:&lt;name&gt;' — fills every row with a value computed at load time. Available functions:
+  fn:now       — current timestamp (timestamp, text)
+  fn:today     — current date (date, text)
+  fn:uuid      — random UUID per row (text)
+  fn:file_name — source file name (text)
+  fn:sequence  — counter 1,2,3... per table (integer, numeric, text)
+4. Expression: 'expr:&lt;expression&gt;' — computes a value from other columns, constants, functions and literals. Use {X} to reference Excel column X.
+  Operators: + - * / (numeric), &amp; (string concatenation)
+  Grouping: parentheses ( ) to override precedence
+  Unary minus: -{A} to negate a value
+  NULL handling: arithmetic with NULL -&gt; NULL (like SQL)
+  Examples:
+    expr:{D} + {E}             (sum two columns)
+    expr:({A} + {B}) * {C}     (grouped arithmetic)
+    expr:-{D}                  (negate a value)
+    expr:{A} &amp; " - " &amp; {C}    (concatenate with separator)
+    expr:{D} * 0.18            (calculate 18% tax)
+All results are cast to the column's data_type. 'script' and
+'null_default' apply after the expression result is cast.
+IMPORTANT: if the supplier inserts a new column, every letter after it shifts. Re-check all col: and expr: source_ref values when that happens.</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>col:&lt;letter&gt;, const:&lt;value&gt;, fn:&lt;name&gt;, or expr:&lt;expression&gt;</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>col:A</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>source_header</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>The header text as printed in the source file — purely for documentation. The parser never matches by header text; it always uses source_ref.
 Example: if column A has header 'Invoice No', put 'Invoice No' here. This shows up in the ER diagram and preview tooltips. If the supplier renames the header, the load still works — only source_ref matters.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>any text; documentation only</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Invoice No</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>column_name</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>The database column name to create. Must be unique within the table.
 Example: 'Invoice No' → 'invoice_no', 'Order Date' → 'order_date'.
 Reserved names (added automatically): file_id, sheet_name, source_row_num, &lt;table_name&gt;_id — do not use these.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>lowercase letters/digits/underscore, unique within the table, max 63 chars</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>invoice_no</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>How the cell value is converted. Choose the type based on the MESSIEST value in the column, not just the first row.
   text     → keeps the text, trims whitespace. Use for names, IDs, mixed content.
@@ -1993,29 +2100,29 @@
 If ANY cell can hold '-', 'NA', or a note, use 'text' to avoid NULLs.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>text | numeric | integer | date | timestamp | boolean</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>nullable</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Can this column be empty in the source?
   Y = empty cells are stored as NULL (most columns should use this).
@@ -2024,86 +2131,86 @@
 When in doubt, use Y — it is safer and you can tighten later.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Y | N</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>is_key</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Creates a non-unique INDEX on this column for faster lookups. This is NOT a primary key and does NOT deduplicate rows.
 Example: set Y on 'order_id' or 'invoice_no' — columns you will filter or join on. Set N on 'amount', 'description', etc.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Y | N</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>column_order</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Controls the position of this column in the created table. Number them 1, 2, 3... in the order you want.
 Example: invoice_no=1, invoice_date=2, customer=3, amount=4.
 Gaps are fine (1, 5, 10); duplicates make the order arbitrary.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>whole number</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>script</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Transformations applied AFTER type casting on every cell value. Chain multiple with | (pipe).
 TEXT examples:
@@ -2140,85 +2247,85 @@
   not_empty        error if NULL or empty string</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>chain with |, e.g. trim|uppercase</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>trim</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>What this column represents. Written as a COMMENT ON COLUMN in PostgreSQL so BI tools and AI agents can understand the schema.
 Example: 'Unique order identifier assigned by the platform'</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>any text</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Unique order identifier from the platform</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Unit of measurement for numeric columns. Appended to the column comment.
 Example: 'INR' for Indian Rupees, 'USD', 'percent', 'count', 'kg'</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>any text</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>INR</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>null_default</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>What to store when a cell is empty, instead of NULL.
 Examples:
@@ -2228,44 +2335,74 @@
 Applied after type casting, so a cell with '-' that casts to NULL also gets the default. Leave blank to keep NULL (the default behavior).</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>any value appropriate for the data_type; blank = store NULL</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>references</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Declares a foreign-key relationship to another table's column. Shown as a dashed line in the ER diagram. Does NOT create a database constraint — it is for documentation and the diagram only.
 Example: if this column references the 'order_id' column in the 'orders' table, write 'orders.order_id'. The ER diagram will draw an arrow from this column to orders.order_id.</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>table_name.column_name (must reference an existing table and column)</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>orders.order_id</t>
         </is>
       </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>date_format</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Pin the date parsing to a specific format instead of auto-detecting.
+Without this, the parser tries multiple formats in order — which means '01/02/2026' could be January 2 or February 1 depending on which format matches first.
+Set this to eliminate ambiguity:
+  %d/%m/%Y   → DD/MM/YYYY (European/Indian: 01/02/2026 = Feb 1)
+  %m/%d/%Y   → MM/DD/YYYY (American: 01/02/2026 = Jan 2)
+  %Y-%m-%d   → YYYY-MM-DD (ISO)
+  %d-%b-%Y   → DD-Mon-YYYY (02-Aug-2026)
+Only applies to date and timestamp columns. Ignored for other types.</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Python strptime format string; blank = auto-detect</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2281,150 +2418,150 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" style="3" min="1" max="1"/>
+    <col width="70" customWidth="1" style="3" min="2" max="2"/>
+    <col width="52" customWidth="1" style="3" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>data_type - what the loader does to the cell value</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>data_type</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>conversion</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>example</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>trimmed; an empty cell becomes NULL</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>" VISA "  -&gt;  VISA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>numeric</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>keeps digits, . and -; a bracketed value becomes negative</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>₹1,234.50 -&gt; 1234.5   18% -&gt; 18.0   (₹120.00) -&gt; -120.0</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>integer</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>as numeric, then cut to a whole number</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>"42.0"  -&gt;  42</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Excel dates and common text dates -&gt; YYYY-MM-DD; '-' and 'NA' -&gt; NULL; anything else -&gt; NULL and reported</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>02-08-2026  -&gt;  2026-08-02</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>timestamp</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>as date, keeping the time</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>2026-08-02 19:45  -&gt;  2026-08-02T19:45</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>boolean</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>y/yes/true/1 -&gt; 1, n/no/false/0 -&gt; 0, anything else NULL</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Yes  -&gt;  1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>A value that does not fit its type is stored as NULL and listed at the end of the load - fix the data_type when you see that.</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
-      <c r="C11" s="4" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>